<commit_message>
Use example products instead of KK's in the template and placeholders
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SpbCHAykWyiFkvqGrGvqvP
</commit_message>
<xml_diff>
--- a/routine-template.xlsx
+++ b/routine-template.xlsx
@@ -463,12 +463,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Beauty of Joseon</t>
+          <t>Banila Co</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Radiance Cleansing Balm</t>
+          <t>Clean It Zero Cleansing Balm Original</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -509,12 +509,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Beauty of Joseon</t>
+          <t>Hada Labo</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ginseng Essence Water</t>
+          <t>Gokujyun Premium Hydrating Lotion</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -537,7 +537,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2% BHA Liquid Exfoliant</t>
+          <t>Skin Perfecting 2% BHA Liquid Exfoliant</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -559,12 +559,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Round Lab</t>
+          <t>The Ordinary</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Vita Niacinamide Dark Spot Serum</t>
+          <t>Niacinamide 10% + Zinc 1%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -609,12 +609,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CeraVe</t>
+          <t>Etude</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Moisturising Lotion</t>
+          <t>SoonJung 2x Barrier Intensive Cream</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -632,12 +632,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Beauty of Joseon</t>
+          <t>La Roche-Posay</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Relief Sun Aqua-fresh Rice + B5 SPF 50+ PA++++</t>
+          <t>Anthelios UVMune 400 Invisible Fluid SPF 50+</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">

</xml_diff>